<commit_message>
Deploying to gh-pages from @ SVNSreedevi/APP@54983e1dbe32396605ae8415d735f671321f3c48 🚀
</commit_message>
<xml_diff>
--- a/reports/latest/execution-report.xlsx
+++ b/reports/latest/execution-report.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Error Log" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="By Category" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Test Cases" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>Metric</t>
   </si>
@@ -29,25 +30,25 @@
     <t>Failed</t>
   </si>
   <si>
-    <t>Skipped</t>
-  </si>
-  <si>
     <t>Pass Rate (%)</t>
   </si>
   <si>
-    <t>0.00%</t>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Test Title</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>FATAL CRASH</t>
+    <t>Duration (ms)</t>
   </si>
   <si>
     <t>Error</t>
-  </si>
-  <si>
-    <t>WebDriverIO execution failed to complete. See CI logs for details.</t>
   </si>
 </sst>
 </file>
@@ -424,11 +425,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="1" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -460,31 +460,15 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B5" t="s">
         <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -495,19 +479,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="100" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="80" customWidth="1"/>
+    <col min="3" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="E1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>